<commit_message>
Deletd columns preferredSiteAnalysisID	and preferredVelocityProfileID
</commit_message>
<xml_diff>
--- a/obspy/io/sitexml/tests/data/sera_site_no_analysis.xlsx
+++ b/obspy/io/sitexml/tests/data/sera_site_no_analysis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kiriaki/Desktop/ITSAK/ORFEUS/SITEXML/obspy15/obspy/obspy/io/sitexml/tests/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAD36B93-0C7D-7F48-88A9-4659F9E44048}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84630149-4DBC-9542-B3DD-77F3CE195730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17320" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="136">
   <si>
     <t>siteID</t>
   </si>
@@ -203,12 +203,6 @@
     <t>overallQindex</t>
   </si>
   <si>
-    <t>preferredSiteAnalysisID</t>
-  </si>
-  <si>
-    <t>preferredVelocityProfileID</t>
-  </si>
-  <si>
     <t>quakeml:domain.ab/site/001</t>
   </si>
   <si>
@@ -272,12 +266,6 @@
     <t>0.41</t>
   </si>
   <si>
-    <t>quakeml:domain.ab/analysis/001</t>
-  </si>
-  <si>
-    <t>quakeml:domain.ab/velocity_profile/001</t>
-  </si>
-  <si>
     <t>quakeml:domain.ab/site/002</t>
   </si>
   <si>
@@ -321,9 +309,6 @@
   </si>
   <si>
     <t>IGME</t>
-  </si>
-  <si>
-    <t>quakeml:domain.ab/analysis/004</t>
   </si>
   <si>
     <t>ownerID</t>
@@ -1812,126 +1797,126 @@
   <sheetData>
     <row r="1" spans="1:20" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="F1" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="G1" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="H1" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="I1" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="J1" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="K1" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="L1" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="M1" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="N1" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="O1" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="P1" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="L1" s="9" t="s">
+      <c r="Q1" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="M1" s="9" t="s">
+      <c r="R1" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="S1" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="O1" s="9" t="s">
+      <c r="T1" s="9" t="s">
         <v>115</v>
-      </c>
-      <c r="P1" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="Q1" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="R1" s="9" t="s">
-        <v>118</v>
-      </c>
-      <c r="S1" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="T1" s="9" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="16" t="s">
+        <v>116</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="F2" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="G2" s="13" t="s">
         <v>122</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="H2" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="I2" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="J2" s="12" t="s">
         <v>125</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="K2" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="L2" s="14" t="s">
         <v>127</v>
       </c>
-      <c r="H2" s="12" t="s">
+      <c r="M2" s="12" t="s">
         <v>128</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="N2" s="12" t="s">
         <v>129</v>
       </c>
-      <c r="J2" s="12" t="s">
+      <c r="O2" s="12" t="s">
         <v>130</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="L2" s="14" t="s">
-        <v>132</v>
-      </c>
-      <c r="M2" s="12" t="s">
-        <v>133</v>
-      </c>
-      <c r="N2" s="12" t="s">
-        <v>134</v>
-      </c>
-      <c r="O2" s="12" t="s">
-        <v>135</v>
       </c>
       <c r="P2" s="15">
         <v>12345</v>
       </c>
       <c r="Q2" s="12" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="R2" s="12" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="S2" s="12" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="T2" s="12" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -1952,15 +1937,15 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BJ3"/>
+  <dimension ref="A1:BH3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="16.33203125" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="9" width="16.33203125" customWidth="1"/>
     <col min="10" max="10" width="19.6640625" customWidth="1"/>
-    <col min="11" max="64" width="16.33203125" customWidth="1"/>
+    <col min="11" max="62" width="16.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:62" ht="32.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:60" ht="32.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2141,28 +2126,22 @@
       <c r="BH1" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="BI1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:60" ht="128.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A2" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="BJ1" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="2" spans="1:62" ht="128.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="2" t="s">
+      <c r="C2" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="E2" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>66</v>
       </c>
       <c r="F2" s="3">
         <v>239</v>
@@ -2170,35 +2149,35 @@
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
       <c r="I2" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="J2" s="3">
         <v>1</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M2" s="3"/>
       <c r="N2" s="2">
         <v>2018</v>
       </c>
       <c r="O2" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="P2" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="Q2" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="P2" s="6" t="s">
+      <c r="R2" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="Q2" s="2" t="s">
+      <c r="S2" s="6" t="s">
         <v>72</v>
-      </c>
-      <c r="R2" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="S2" s="6" t="s">
-        <v>74</v>
       </c>
       <c r="T2" s="3">
         <v>40</v>
@@ -2207,7 +2186,7 @@
         <v>6</v>
       </c>
       <c r="V2" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="W2" s="3"/>
       <c r="X2" s="3"/>
@@ -2225,13 +2204,13 @@
         <v>1</v>
       </c>
       <c r="AH2" s="6" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="AI2" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="AJ2" s="6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="AK2" s="3"/>
       <c r="AL2" s="2"/>
@@ -2241,72 +2220,66 @@
       <c r="AP2" s="3"/>
       <c r="AQ2" s="3"/>
       <c r="AR2" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="AS2" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="AT2" s="3"/>
       <c r="AU2" s="3"/>
       <c r="AV2" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="AW2" s="6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="AX2" s="3"/>
       <c r="AY2" s="2">
         <v>2018</v>
       </c>
       <c r="AZ2" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="BA2" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="BB2" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="BA2" s="6" t="s">
+      <c r="BC2" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="BB2" s="2" t="s">
+      <c r="BD2" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="BC2" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="BD2" s="6" t="s">
-        <v>74</v>
-      </c>
       <c r="BE2" s="6" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="BF2" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="BG2" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="BH2" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="BG2" s="2" t="s">
+    </row>
+    <row r="3" spans="1:60" ht="44" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A3" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="BH2" s="2" t="s">
+      <c r="B3" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="BI2" s="2" t="s">
+      <c r="C3" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="BJ2" s="6" t="s">
+      <c r="D3" s="4" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="3" spans="1:62" ht="44" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="4" t="s">
+      <c r="E3" s="4" t="s">
         <v>85</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>89</v>
       </c>
       <c r="F3" s="5">
         <v>120</v>
@@ -2314,33 +2287,33 @@
       <c r="G3" s="5"/>
       <c r="H3" s="5"/>
       <c r="I3" s="7" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="J3" s="5">
         <v>1</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="L3" s="7" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="M3" s="5"/>
       <c r="N3" s="2">
         <v>2023</v>
       </c>
       <c r="O3" s="8" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="P3" s="8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="Q3" s="7" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="R3" s="5"/>
       <c r="S3" s="4" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="T3" s="5">
         <v>820</v>
@@ -2350,27 +2323,27 @@
         <v>0.8</v>
       </c>
       <c r="W3" s="2" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="X3" s="7" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="Y3" s="5"/>
       <c r="Z3" s="2">
         <v>2023</v>
       </c>
       <c r="AA3" s="8" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="AB3" s="8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="AC3" s="7" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="AD3" s="5"/>
       <c r="AE3" s="4" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="AF3" s="5">
         <v>180</v>
@@ -2378,41 +2351,41 @@
       <c r="AG3" s="5"/>
       <c r="AH3" s="5"/>
       <c r="AI3" s="2" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="AJ3" s="7" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="AK3" s="5"/>
       <c r="AL3" s="2">
         <v>2023</v>
       </c>
       <c r="AM3" s="8" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="AN3" s="8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="AO3" s="7" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="AP3" s="5"/>
       <c r="AQ3" s="4" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="AR3" s="4" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="AS3" s="5"/>
       <c r="AT3" s="4" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="AU3" s="5"/>
       <c r="AV3" s="4" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="AW3" s="4" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="AX3" s="5"/>
       <c r="AY3" s="2"/>
@@ -2425,12 +2398,6 @@
       <c r="BF3" s="5"/>
       <c r="BG3" s="5"/>
       <c r="BH3" s="5"/>
-      <c r="BI3" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="BJ3" s="4" t="s">
-        <v>100</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>

</xml_diff>